<commit_message>
Add poster draft and full pipeline re-run artefacts
Refresh outputs from running R/*.R end-to-end (run_all.R) to verify
reproducibility, regenerate missing PCA/integrated-analysis outputs
that were not previously committed, and add a structured poster
draft (reports/poster_draft.md) covering the LASSO/parsimonious/LMM
pipeline, spatial diagnostics and PCR/PLS comparison.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/pca/tables/PCA_Threshold_Summary.xlsx
+++ b/outputs/pca/tables/PCA_Threshold_Summary.xlsx
@@ -1,162 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11110"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shuvroahmed/Desktop/Imaging Program Academics/POLIMI/sem 2/applied stat/projects/PCA_Presentation_Output/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8708FA2-053E-E64F-88B0-CEEAE2200382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Threshold_Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Explained_Long" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="43">
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>PCs_Needed_for_70pct</t>
-  </si>
-  <si>
-    <t>Cumulative_at_70pct</t>
-  </si>
-  <si>
-    <t>Breakdown_to_70pct</t>
-  </si>
-  <si>
-    <t>PCs_Needed_for_80pct</t>
-  </si>
-  <si>
-    <t>Cumulative_at_80pct</t>
-  </si>
-  <si>
-    <t>Breakdown_to_80pct</t>
-  </si>
-  <si>
-    <t>PC1_Pct</t>
-  </si>
-  <si>
-    <t>PC2_Pct</t>
-  </si>
-  <si>
-    <t>PC3_Pct</t>
-  </si>
-  <si>
-    <t>PC4_Pct</t>
-  </si>
-  <si>
-    <t>PC5_Pct</t>
-  </si>
-  <si>
-    <t>PC6_Pct</t>
-  </si>
-  <si>
-    <t>2018</t>
-  </si>
-  <si>
-    <t>PC1=29.19% | PC2=13.77% | PC3=9.09% | PC4=8.14% | PC5=6.95% | PC6=6.94%</t>
-  </si>
-  <si>
-    <t>PC1=29.19% | PC2=13.77% | PC3=9.09% | PC4=8.14% | PC5=6.95% | PC6=6.94% | PC7=6.52%</t>
-  </si>
-  <si>
-    <t>2019</t>
-  </si>
-  <si>
-    <t>PC1=29.21% | PC2=13.88% | PC3=8.98% | PC4=8.05% | PC5=6.96% | PC6=6.85%</t>
-  </si>
-  <si>
-    <t>PC1=29.21% | PC2=13.88% | PC3=8.98% | PC4=8.05% | PC5=6.96% | PC6=6.85% | PC7=6.41%</t>
-  </si>
-  <si>
-    <t>2021</t>
-  </si>
-  <si>
-    <t>PC1=29.8% | PC2=13.93% | PC3=8.45% | PC4=7.97% | PC5=7.01% | PC6=6.9%</t>
-  </si>
-  <si>
-    <t>PC1=29.8% | PC2=13.93% | PC3=8.45% | PC4=7.97% | PC5=7.01% | PC6=6.9% | PC7=6.49%</t>
-  </si>
-  <si>
-    <t>2022</t>
-  </si>
-  <si>
-    <t>PC1=30.07% | PC2=14.17% | PC3=8.45% | PC4=7.8% | PC5=7.06% | PC6=6.76%</t>
-  </si>
-  <si>
-    <t>PC1=30.07% | PC2=14.17% | PC3=8.45% | PC4=7.8% | PC5=7.06% | PC6=6.76% | PC7=6.44%</t>
-  </si>
-  <si>
-    <t>PC</t>
-  </si>
-  <si>
-    <t>Variance_Explained</t>
-  </si>
-  <si>
-    <t>Cumulative_Variance</t>
-  </si>
-  <si>
-    <t>PC_num</t>
-  </si>
-  <si>
-    <t>Variance_Explained_Pct</t>
-  </si>
-  <si>
-    <t>Cumulative_Variance_Pct</t>
-  </si>
-  <si>
-    <t>PC1</t>
-  </si>
-  <si>
-    <t>PC2</t>
-  </si>
-  <si>
-    <t>PC3</t>
-  </si>
-  <si>
-    <t>PC4</t>
-  </si>
-  <si>
-    <t>PC5</t>
-  </si>
-  <si>
-    <t>PC6</t>
-  </si>
-  <si>
-    <t>PC7</t>
-  </si>
-  <si>
-    <t>PC8</t>
-  </si>
-  <si>
-    <t>PC9</t>
-  </si>
-  <si>
-    <t>PC10</t>
-  </si>
-  <si>
-    <t>PC11</t>
-  </si>
-  <si>
-    <t>PC12</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -204,21 +64,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -256,7 +108,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -290,7 +142,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -325,10 +176,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -501,54 +351,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>13</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PCs_Needed_for_70pct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cumulative_at_70pct</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Breakdown_to_70pct</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PCs_Needed_for_80pct</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Cumulative_at_80pct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Breakdown_to_80pct</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>PC1_Pct</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>PC2_Pct</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>PC3_Pct</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>PC4_Pct</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>PC5_Pct</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>PC6_Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="B2">
         <v>6</v>
@@ -556,17 +434,21 @@
       <c r="C2">
         <v>74.08</v>
       </c>
-      <c r="D2" t="s">
-        <v>14</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PC1=29.19% | PC2=13.77% | PC3=9.09% | PC4=8.14% | PC5=6.95% | PC6=6.94%</t>
+        </is>
       </c>
       <c r="E2">
         <v>7</v>
       </c>
       <c r="F2">
-        <v>80.599999999999994</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
+        <v>80.59999999999999</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PC1=29.19% | PC2=13.77% | PC3=9.09% | PC4=8.14% | PC5=6.95% | PC6=6.94% | PC7=6.52%</t>
+        </is>
       </c>
       <c r="H2">
         <v>29.19</v>
@@ -578,7 +460,7 @@
         <v>9.09</v>
       </c>
       <c r="K2">
-        <v>8.14</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="L2">
         <v>6.95</v>
@@ -587,27 +469,33 @@
         <v>6.94</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>16</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="B3">
         <v>6</v>
       </c>
       <c r="C3">
-        <v>73.930000000000007</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
+        <v>73.93000000000001</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PC1=29.21% | PC2=13.88% | PC3=8.98% | PC4=8.05% | PC5=6.96% | PC6=6.85%</t>
+        </is>
       </c>
       <c r="E3">
         <v>7</v>
       </c>
       <c r="F3">
-        <v>80.349999999999994</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
+        <v>80.34999999999999</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PC1=29.21% | PC2=13.88% | PC3=8.98% | PC4=8.05% | PC5=6.96% | PC6=6.85% | PC7=6.41%</t>
+        </is>
       </c>
       <c r="H3">
         <v>29.21</v>
@@ -619,7 +507,7 @@
         <v>8.98</v>
       </c>
       <c r="K3">
-        <v>8.0500000000000007</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="L3">
         <v>6.96</v>
@@ -628,9 +516,11 @@
         <v>6.85</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>19</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="B4">
         <v>6</v>
@@ -638,8 +528,10 @@
       <c r="C4">
         <v>74.06</v>
       </c>
-      <c r="D4" t="s">
-        <v>20</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PC1=29.8% | PC2=13.93% | PC3=8.45% | PC4=7.97% | PC5=7.01% | PC6=6.9%</t>
+        </is>
       </c>
       <c r="E4">
         <v>7</v>
@@ -647,8 +539,10 @@
       <c r="F4">
         <v>80.55</v>
       </c>
-      <c r="G4" t="s">
-        <v>21</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PC1=29.8% | PC2=13.93% | PC3=8.45% | PC4=7.97% | PC5=7.01% | PC6=6.9% | PC7=6.49%</t>
+        </is>
       </c>
       <c r="H4">
         <v>29.8</v>
@@ -657,7 +551,7 @@
         <v>13.93</v>
       </c>
       <c r="J4">
-        <v>8.4499999999999993</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="K4">
         <v>7.97</v>
@@ -669,9 +563,11 @@
         <v>6.9</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>22</v>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="B5">
         <v>6</v>
@@ -679,17 +575,21 @@
       <c r="C5">
         <v>74.31</v>
       </c>
-      <c r="D5" t="s">
-        <v>23</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PC1=30.07% | PC2=14.17% | PC3=8.45% | PC4=7.8% | PC5=7.06% | PC6=6.76%</t>
+        </is>
       </c>
       <c r="E5">
         <v>7</v>
       </c>
       <c r="F5">
-        <v>80.739999999999995</v>
-      </c>
-      <c r="G5" t="s">
-        <v>24</v>
+        <v>80.73999999999999</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PC1=30.07% | PC2=14.17% | PC3=8.45% | PC4=7.8% | PC5=7.06% | PC6=6.76% | PC7=6.44%</t>
+        </is>
       </c>
       <c r="H5">
         <v>30.07</v>
@@ -698,7 +598,7 @@
         <v>14.17</v>
       </c>
       <c r="J5">
-        <v>8.4499999999999993</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="K5">
         <v>7.8</v>
@@ -716,45 +616,63 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G49"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>31</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Variance_Explained</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Cumulative_Variance</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PC_num</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Variance_Explained_Pct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Cumulative_Variance_Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PC1</t>
+        </is>
       </c>
       <c r="C2">
-        <v>0.29190461835939652</v>
+        <v>0.2919046183593965</v>
       </c>
       <c r="D2">
-        <v>0.29190461835939652</v>
+        <v>0.2919046183593965</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -766,18 +684,22 @@
         <v>29.19</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PC2</t>
+        </is>
       </c>
       <c r="C3">
         <v>0.1377006329095129</v>
       </c>
       <c r="D3">
-        <v>0.42960525126890942</v>
+        <v>0.4296052512689094</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -789,15 +711,19 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>33</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PC3</t>
+        </is>
       </c>
       <c r="C4">
-        <v>9.0938607461588425E-2</v>
+        <v>0.09093860746158842</v>
       </c>
       <c r="D4">
         <v>0.5205438587304978</v>
@@ -812,41 +738,49 @@
         <v>52.05</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>34</v>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PC4</t>
+        </is>
       </c>
       <c r="C5">
-        <v>8.1356349024178348E-2</v>
+        <v>0.08135634902417835</v>
       </c>
       <c r="D5">
-        <v>0.60190020775467623</v>
+        <v>0.6019002077546762</v>
       </c>
       <c r="E5">
         <v>4</v>
       </c>
       <c r="F5">
-        <v>8.14</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="G5">
         <v>60.19</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>35</v>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PC5</t>
+        </is>
       </c>
       <c r="C6">
-        <v>6.9537264792348244E-2</v>
+        <v>0.06953726479234824</v>
       </c>
       <c r="D6">
-        <v>0.67143747254702446</v>
+        <v>0.6714374725470245</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -858,15 +792,19 @@
         <v>67.14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>36</v>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PC6</t>
+        </is>
       </c>
       <c r="C7">
-        <v>6.9397097804797692E-2</v>
+        <v>0.06939709780479769</v>
       </c>
       <c r="D7">
         <v>0.7408345703518221</v>
@@ -881,15 +819,19 @@
         <v>74.08</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PC7</t>
+        </is>
       </c>
       <c r="C8">
-        <v>6.5212620513813532E-2</v>
+        <v>0.06521262051381353</v>
       </c>
       <c r="D8">
         <v>0.8060471908656357</v>
@@ -901,18 +843,22 @@
         <v>6.52</v>
       </c>
       <c r="G8">
-        <v>80.599999999999994</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>38</v>
+        <v>80.59999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PC8</t>
+        </is>
       </c>
       <c r="C9">
-        <v>5.3825878086749122E-2</v>
+        <v>0.05382587808674912</v>
       </c>
       <c r="D9">
         <v>0.8598730689523848</v>
@@ -924,21 +870,25 @@
         <v>5.38</v>
       </c>
       <c r="G9">
-        <v>85.99</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>39</v>
+        <v>85.98999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PC9</t>
+        </is>
       </c>
       <c r="C10">
-        <v>4.7248602891630319E-2</v>
+        <v>0.04724860289163032</v>
       </c>
       <c r="D10">
-        <v>0.90712167184401515</v>
+        <v>0.9071216718440152</v>
       </c>
       <c r="E10">
         <v>9</v>
@@ -947,21 +897,25 @@
         <v>4.72</v>
       </c>
       <c r="G10">
-        <v>90.71</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
+        <v>90.70999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PC10</t>
+        </is>
       </c>
       <c r="C11">
-        <v>3.9423087865483833E-2</v>
+        <v>0.03942308786548383</v>
       </c>
       <c r="D11">
-        <v>0.94654475970949892</v>
+        <v>0.9465447597094989</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -970,21 +924,25 @@
         <v>3.94</v>
       </c>
       <c r="G11">
-        <v>94.65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>41</v>
+        <v>94.65000000000001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PC11</t>
+        </is>
       </c>
       <c r="C12">
-        <v>3.2414377063096182E-2</v>
+        <v>0.03241437706309618</v>
       </c>
       <c r="D12">
-        <v>0.97895913677259516</v>
+        <v>0.9789591367725952</v>
       </c>
       <c r="E12">
         <v>11</v>
@@ -993,21 +951,25 @@
         <v>3.24</v>
       </c>
       <c r="G12">
-        <v>97.9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
-        <v>42</v>
+        <v>97.90000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PC12</t>
+        </is>
       </c>
       <c r="C13">
-        <v>2.1040863227404821E-2</v>
+        <v>0.02104086322740482</v>
       </c>
       <c r="D13">
-        <v>0.99999999999999989</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="E13">
         <v>12</v>
@@ -1019,18 +981,22 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" t="s">
-        <v>31</v>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PC1</t>
+        </is>
       </c>
       <c r="C14">
-        <v>0.29212121280101888</v>
+        <v>0.2921212128010189</v>
       </c>
       <c r="D14">
-        <v>0.29212121280101888</v>
+        <v>0.2921212128010189</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -1042,18 +1008,22 @@
         <v>29.21</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" t="s">
-        <v>32</v>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PC2</t>
+        </is>
       </c>
       <c r="C15">
-        <v>0.13879232989048521</v>
+        <v>0.1387923298904852</v>
       </c>
       <c r="D15">
-        <v>0.43091354269150423</v>
+        <v>0.4309135426915042</v>
       </c>
       <c r="E15">
         <v>2</v>
@@ -1065,18 +1035,22 @@
         <v>43.09</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" t="s">
-        <v>33</v>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PC3</t>
+        </is>
       </c>
       <c r="C16">
-        <v>8.9775002365288264E-2</v>
+        <v>0.08977500236528826</v>
       </c>
       <c r="D16">
-        <v>0.52068854505679241</v>
+        <v>0.5206885450567924</v>
       </c>
       <c r="E16">
         <v>3</v>
@@ -1088,41 +1062,49 @@
         <v>52.07</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>34</v>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PC4</t>
+        </is>
       </c>
       <c r="C17">
-        <v>8.0472574320202162E-2</v>
+        <v>0.08047257432020216</v>
       </c>
       <c r="D17">
-        <v>0.60116111937699457</v>
+        <v>0.6011611193769946</v>
       </c>
       <c r="E17">
         <v>4</v>
       </c>
       <c r="F17">
-        <v>8.0500000000000007</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="G17">
         <v>60.12</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PC5</t>
+        </is>
       </c>
       <c r="C18">
-        <v>6.9629294077631021E-2</v>
+        <v>0.06962929407763102</v>
       </c>
       <c r="D18">
-        <v>0.67079041345462564</v>
+        <v>0.6707904134546256</v>
       </c>
       <c r="E18">
         <v>5</v>
@@ -1134,18 +1116,22 @@
         <v>67.08</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19" t="s">
-        <v>36</v>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PC6</t>
+        </is>
       </c>
       <c r="C19">
-        <v>6.8541313335651805E-2</v>
+        <v>0.0685413133356518</v>
       </c>
       <c r="D19">
-        <v>0.73933172679027748</v>
+        <v>0.7393317267902775</v>
       </c>
       <c r="E19">
         <v>6</v>
@@ -1154,21 +1140,25 @@
         <v>6.85</v>
       </c>
       <c r="G19">
-        <v>73.930000000000007</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" t="s">
-        <v>37</v>
+        <v>73.93000000000001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PC7</t>
+        </is>
       </c>
       <c r="C20">
-        <v>6.4138616895900946E-2</v>
+        <v>0.06413861689590095</v>
       </c>
       <c r="D20">
-        <v>0.80347034368617831</v>
+        <v>0.8034703436861783</v>
       </c>
       <c r="E20">
         <v>7</v>
@@ -1177,21 +1167,25 @@
         <v>6.41</v>
       </c>
       <c r="G20">
-        <v>80.349999999999994</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" t="s">
-        <v>38</v>
+        <v>80.34999999999999</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PC8</t>
+        </is>
       </c>
       <c r="C21">
-        <v>5.415393465034489E-2</v>
+        <v>0.05415393465034489</v>
       </c>
       <c r="D21">
-        <v>0.85762427833652322</v>
+        <v>0.8576242783365232</v>
       </c>
       <c r="E21">
         <v>8</v>
@@ -1200,44 +1194,52 @@
         <v>5.42</v>
       </c>
       <c r="G21">
-        <v>85.76</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>16</v>
-      </c>
-      <c r="B22" t="s">
-        <v>39</v>
+        <v>85.76000000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PC9</t>
+        </is>
       </c>
       <c r="C22">
-        <v>4.7699065034316521E-2</v>
+        <v>0.04769906503431652</v>
       </c>
       <c r="D22">
-        <v>0.90532334337083975</v>
+        <v>0.9053233433708398</v>
       </c>
       <c r="E22">
         <v>9</v>
       </c>
       <c r="F22">
-        <v>4.7699999999999996</v>
+        <v>4.77</v>
       </c>
       <c r="G22">
         <v>90.53</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>16</v>
-      </c>
-      <c r="B23" t="s">
-        <v>40</v>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PC10</t>
+        </is>
       </c>
       <c r="C23">
-        <v>3.9843640929372023E-2</v>
+        <v>0.03984364092937202</v>
       </c>
       <c r="D23">
-        <v>0.94516698430021184</v>
+        <v>0.9451669843002118</v>
       </c>
       <c r="E23">
         <v>10</v>
@@ -1249,18 +1251,22 @@
         <v>94.52</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>16</v>
-      </c>
-      <c r="B24" t="s">
-        <v>41</v>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PC11</t>
+        </is>
       </c>
       <c r="C24">
-        <v>3.3324514582236731E-2</v>
+        <v>0.03332451458223673</v>
       </c>
       <c r="D24">
-        <v>0.97849149888244857</v>
+        <v>0.9784914988824486</v>
       </c>
       <c r="E24">
         <v>11</v>
@@ -1269,18 +1275,22 @@
         <v>3.33</v>
       </c>
       <c r="G24">
-        <v>97.85</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" t="s">
-        <v>42</v>
+        <v>97.84999999999999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PC12</t>
+        </is>
       </c>
       <c r="C25">
-        <v>2.1508501117551499E-2</v>
+        <v>0.0215085011175515</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -1295,18 +1305,22 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" t="s">
-        <v>31</v>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PC1</t>
+        </is>
       </c>
       <c r="C26">
-        <v>0.29803050963411798</v>
+        <v>0.298030509634118</v>
       </c>
       <c r="D26">
-        <v>0.29803050963411798</v>
+        <v>0.298030509634118</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -1318,18 +1332,22 @@
         <v>29.8</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" t="s">
-        <v>32</v>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PC2</t>
+        </is>
       </c>
       <c r="C27">
-        <v>0.13928989740862929</v>
+        <v>0.1392898974086293</v>
       </c>
       <c r="D27">
-        <v>0.43732040704274727</v>
+        <v>0.4373204070427473</v>
       </c>
       <c r="E27">
         <v>2</v>
@@ -1341,41 +1359,49 @@
         <v>43.73</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" t="s">
-        <v>33</v>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PC3</t>
+        </is>
       </c>
       <c r="C28">
-        <v>8.4521559871055557E-2</v>
+        <v>0.08452155987105556</v>
       </c>
       <c r="D28">
-        <v>0.52184196691380291</v>
+        <v>0.5218419669138029</v>
       </c>
       <c r="E28">
         <v>3</v>
       </c>
       <c r="F28">
-        <v>8.4499999999999993</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="G28">
         <v>52.18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" t="s">
-        <v>34</v>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PC4</t>
+        </is>
       </c>
       <c r="C29">
-        <v>7.9660639527625962E-2</v>
+        <v>0.07966063952762596</v>
       </c>
       <c r="D29">
-        <v>0.60150260644142883</v>
+        <v>0.6015026064414288</v>
       </c>
       <c r="E29">
         <v>4</v>
@@ -1387,18 +1413,22 @@
         <v>60.15</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>19</v>
-      </c>
-      <c r="B30" t="s">
-        <v>35</v>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PC5</t>
+        </is>
       </c>
       <c r="C30">
-        <v>7.0114871979755494E-2</v>
+        <v>0.07011487197975549</v>
       </c>
       <c r="D30">
-        <v>0.67161747842118436</v>
+        <v>0.6716174784211844</v>
       </c>
       <c r="E30">
         <v>5</v>
@@ -1410,18 +1440,22 @@
         <v>67.16</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>19</v>
-      </c>
-      <c r="B31" t="s">
-        <v>36</v>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PC6</t>
+        </is>
       </c>
       <c r="C31">
-        <v>6.8999587964643935E-2</v>
+        <v>0.06899958796464394</v>
       </c>
       <c r="D31">
-        <v>0.74061706638582825</v>
+        <v>0.7406170663858282</v>
       </c>
       <c r="E31">
         <v>6</v>
@@ -1433,18 +1467,22 @@
         <v>74.06</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>19</v>
-      </c>
-      <c r="B32" t="s">
-        <v>37</v>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PC7</t>
+        </is>
       </c>
       <c r="C32">
-        <v>6.4891569019765824E-2</v>
+        <v>0.06489156901976582</v>
       </c>
       <c r="D32">
-        <v>0.80550863540559414</v>
+        <v>0.8055086354055941</v>
       </c>
       <c r="E32">
         <v>7</v>
@@ -1456,18 +1494,22 @@
         <v>80.55</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>19</v>
-      </c>
-      <c r="B33" t="s">
-        <v>38</v>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PC8</t>
+        </is>
       </c>
       <c r="C33">
-        <v>5.4747262597712343E-2</v>
+        <v>0.05474726259771234</v>
       </c>
       <c r="D33">
-        <v>0.86025589800330649</v>
+        <v>0.8602558980033065</v>
       </c>
       <c r="E33">
         <v>8</v>
@@ -1479,18 +1521,22 @@
         <v>86.03</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>19</v>
-      </c>
-      <c r="B34" t="s">
-        <v>39</v>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PC9</t>
+        </is>
       </c>
       <c r="C34">
-        <v>4.6810053079009449E-2</v>
+        <v>0.04681005307900945</v>
       </c>
       <c r="D34">
-        <v>0.90706595108231591</v>
+        <v>0.9070659510823159</v>
       </c>
       <c r="E34">
         <v>9</v>
@@ -1499,21 +1545,25 @@
         <v>4.68</v>
       </c>
       <c r="G34">
-        <v>90.71</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>19</v>
-      </c>
-      <c r="B35" t="s">
-        <v>40</v>
+        <v>90.70999999999999</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PC10</t>
+        </is>
       </c>
       <c r="C35">
-        <v>3.945514211343195E-2</v>
+        <v>0.03945514211343195</v>
       </c>
       <c r="D35">
-        <v>0.94652109319574784</v>
+        <v>0.9465210931957478</v>
       </c>
       <c r="E35">
         <v>10</v>
@@ -1522,21 +1572,25 @@
         <v>3.95</v>
       </c>
       <c r="G35">
-        <v>94.65</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>19</v>
-      </c>
-      <c r="B36" t="s">
-        <v>41</v>
+        <v>94.65000000000001</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>PC11</t>
+        </is>
       </c>
       <c r="C36">
-        <v>3.373203297966447E-2</v>
+        <v>0.03373203297966447</v>
       </c>
       <c r="D36">
-        <v>0.98025312617541227</v>
+        <v>0.9802531261754123</v>
       </c>
       <c r="E36">
         <v>11</v>
@@ -1548,15 +1602,19 @@
         <v>98.03</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>19</v>
-      </c>
-      <c r="B37" t="s">
-        <v>42</v>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>PC12</t>
+        </is>
       </c>
       <c r="C37">
-        <v>1.974687382458775E-2</v>
+        <v>0.01974687382458775</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1571,18 +1629,22 @@
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>22</v>
-      </c>
-      <c r="B38" t="s">
-        <v>31</v>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>PC1</t>
+        </is>
       </c>
       <c r="C38">
-        <v>0.30074984742813321</v>
+        <v>0.3007498474281332</v>
       </c>
       <c r="D38">
-        <v>0.30074984742813321</v>
+        <v>0.3007498474281332</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -1594,18 +1656,22 @@
         <v>30.07</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>22</v>
-      </c>
-      <c r="B39" t="s">
-        <v>32</v>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PC2</t>
+        </is>
       </c>
       <c r="C39">
-        <v>0.14173498565518239</v>
+        <v>0.1417349856551824</v>
       </c>
       <c r="D39">
-        <v>0.44248483308331571</v>
+        <v>0.4424848330833157</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -1617,41 +1683,49 @@
         <v>44.25</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>22</v>
-      </c>
-      <c r="B40" t="s">
-        <v>33</v>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PC3</t>
+        </is>
       </c>
       <c r="C40">
-        <v>8.4465963955357853E-2</v>
+        <v>0.08446596395535785</v>
       </c>
       <c r="D40">
-        <v>0.52695079703867354</v>
+        <v>0.5269507970386735</v>
       </c>
       <c r="E40">
         <v>3</v>
       </c>
       <c r="F40">
-        <v>8.4499999999999993</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="G40">
         <v>52.7</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>22</v>
-      </c>
-      <c r="B41" t="s">
-        <v>34</v>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PC4</t>
+        </is>
       </c>
       <c r="C41">
-        <v>7.7992648509275078E-2</v>
+        <v>0.07799264850927508</v>
       </c>
       <c r="D41">
-        <v>0.60494344554794854</v>
+        <v>0.6049434455479485</v>
       </c>
       <c r="E41">
         <v>4</v>
@@ -1663,18 +1737,22 @@
         <v>60.49</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B42" t="s">
-        <v>35</v>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>PC5</t>
+        </is>
       </c>
       <c r="C42">
-        <v>7.0559137707141131E-2</v>
+        <v>0.07055913770714113</v>
       </c>
       <c r="D42">
-        <v>0.67550258325508972</v>
+        <v>0.6755025832550897</v>
       </c>
       <c r="E42">
         <v>5</v>
@@ -1686,18 +1764,22 @@
         <v>67.55</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>22</v>
-      </c>
-      <c r="B43" t="s">
-        <v>36</v>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PC6</t>
+        </is>
       </c>
       <c r="C43">
-        <v>6.7572277875724979E-2</v>
+        <v>0.06757227787572498</v>
       </c>
       <c r="D43">
-        <v>0.74307486113081467</v>
+        <v>0.7430748611308147</v>
       </c>
       <c r="E43">
         <v>6</v>
@@ -1709,18 +1791,22 @@
         <v>74.31</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>22</v>
-      </c>
-      <c r="B44" t="s">
-        <v>37</v>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PC7</t>
+        </is>
       </c>
       <c r="C44">
-        <v>6.4369345194057542E-2</v>
+        <v>0.06436934519405754</v>
       </c>
       <c r="D44">
-        <v>0.80744420632487224</v>
+        <v>0.8074442063248722</v>
       </c>
       <c r="E44">
         <v>7</v>
@@ -1729,21 +1815,25 @@
         <v>6.44</v>
       </c>
       <c r="G44">
-        <v>80.739999999999995</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>22</v>
-      </c>
-      <c r="B45" t="s">
-        <v>38</v>
+        <v>80.73999999999999</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>PC8</t>
+        </is>
       </c>
       <c r="C45">
-        <v>5.345975843310001E-2</v>
+        <v>0.05345975843310001</v>
       </c>
       <c r="D45">
-        <v>0.86090396475797226</v>
+        <v>0.8609039647579723</v>
       </c>
       <c r="E45">
         <v>8</v>
@@ -1755,41 +1845,49 @@
         <v>86.09</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>22</v>
-      </c>
-      <c r="B46" t="s">
-        <v>39</v>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>PC9</t>
+        </is>
       </c>
       <c r="C46">
-        <v>4.6903086103804462E-2</v>
+        <v>0.04690308610380446</v>
       </c>
       <c r="D46">
-        <v>0.90780705086177671</v>
+        <v>0.9078070508617767</v>
       </c>
       <c r="E46">
         <v>9</v>
       </c>
       <c r="F46">
-        <v>4.6900000000000004</v>
+        <v>4.69</v>
       </c>
       <c r="G46">
         <v>90.78</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>22</v>
-      </c>
-      <c r="B47" t="s">
-        <v>40</v>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>PC10</t>
+        </is>
       </c>
       <c r="C47">
-        <v>3.9238306568095419E-2</v>
+        <v>0.03923830656809542</v>
       </c>
       <c r="D47">
-        <v>0.94704535742987217</v>
+        <v>0.9470453574298722</v>
       </c>
       <c r="E47">
         <v>10</v>
@@ -1801,18 +1899,22 @@
         <v>94.7</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>22</v>
-      </c>
-      <c r="B48" t="s">
-        <v>41</v>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>PC11</t>
+        </is>
       </c>
       <c r="C48">
-        <v>3.2787747521894207E-2</v>
+        <v>0.03278774752189421</v>
       </c>
       <c r="D48">
-        <v>0.97983310495176634</v>
+        <v>0.9798331049517663</v>
       </c>
       <c r="E48">
         <v>11</v>
@@ -1824,15 +1926,19 @@
         <v>97.98</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>22</v>
-      </c>
-      <c r="B49" t="s">
-        <v>42</v>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>PC12</t>
+        </is>
       </c>
       <c r="C49">
-        <v>2.0166895048233661E-2</v>
+        <v>0.02016689504823366</v>
       </c>
       <c r="D49">
         <v>1</v>

</xml_diff>